<commit_message>
Atualiza app RDO: equip/veiculos unificados+abreviados, assinatura travada por padrao, lembrar ultima obra, BETA 0.1.0
</commit_message>
<xml_diff>
--- a/assets/modelo_rdo.xlsx
+++ b/assets/modelo_rdo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TecnicoFn01\.local\bin\scripts\rdo_app\www\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{966258D6-1776-40DD-A7A6-D064CF82787F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A97AEE97-BD29-4353-BFFB-06128294229C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5610" yWindow="3225" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -183,7 +183,7 @@
     <t xml:space="preserve">        Responsável da Contratante</t>
   </si>
   <si>
-    <t>Modelo v. beta 1.0.1</t>
+    <t>Modelo v. beta 1.0.2</t>
   </si>
 </sst>
 </file>
@@ -778,6 +778,14 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -787,14 +795,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -804,7 +804,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -813,7 +813,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2178,22 +2178,22 @@
       <c r="A14" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="27" t="s">
+      <c r="B14" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="27" t="s">
+      <c r="E14" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="F14" s="27" t="s">
+      <c r="F14" s="31" t="s">
         <v>36</v>
       </c>
-      <c r="G14" s="27" t="s">
+      <c r="G14" s="31" t="s">
         <v>37</v>
       </c>
       <c r="H14" s="11" t="s">
@@ -2663,17 +2663,17 @@
         <v>21</v>
       </c>
       <c r="B32" s="124"/>
-      <c r="C32" s="29" t="s">
+      <c r="C32" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="D32" s="30" t="s">
+      <c r="D32" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="E32" s="31" t="s">
+      <c r="E32" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="F32" s="32"/>
-      <c r="G32" s="32"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
       <c r="H32" s="13"/>
       <c r="I32" s="13"/>
       <c r="J32" s="13"/>
@@ -2723,8 +2723,8 @@
       <c r="B34" s="25">
         <v>2</v>
       </c>
-      <c r="C34" s="26"/>
-      <c r="D34" s="28"/>
+      <c r="C34" s="30"/>
+      <c r="D34" s="32"/>
       <c r="E34" s="126"/>
       <c r="F34" s="126"/>
       <c r="G34" s="126"/>
@@ -2749,8 +2749,8 @@
       <c r="B35" s="25">
         <v>3</v>
       </c>
-      <c r="C35" s="26"/>
-      <c r="D35" s="28"/>
+      <c r="C35" s="30"/>
+      <c r="D35" s="32"/>
       <c r="E35" s="126"/>
       <c r="F35" s="126"/>
       <c r="G35" s="126"/>
@@ -2775,8 +2775,8 @@
       <c r="B36" s="25">
         <v>4</v>
       </c>
-      <c r="C36" s="26"/>
-      <c r="D36" s="28"/>
+      <c r="C36" s="30"/>
+      <c r="D36" s="32"/>
       <c r="E36" s="126"/>
       <c r="F36" s="126"/>
       <c r="G36" s="126"/>
@@ -2801,8 +2801,8 @@
       <c r="B37" s="25">
         <v>5</v>
       </c>
-      <c r="C37" s="26"/>
-      <c r="D37" s="28"/>
+      <c r="C37" s="30"/>
+      <c r="D37" s="32"/>
       <c r="E37" s="126"/>
       <c r="F37" s="126"/>
       <c r="G37" s="126"/>
@@ -2833,8 +2833,8 @@
       <c r="B38" s="25">
         <v>6</v>
       </c>
-      <c r="C38" s="28"/>
-      <c r="D38" s="28"/>
+      <c r="C38" s="32"/>
+      <c r="D38" s="32"/>
       <c r="E38" s="104"/>
       <c r="F38" s="104"/>
       <c r="G38" s="104"/>
@@ -2865,8 +2865,8 @@
       <c r="B39" s="25">
         <v>7</v>
       </c>
-      <c r="C39" s="28"/>
-      <c r="D39" s="28"/>
+      <c r="C39" s="32"/>
+      <c r="D39" s="32"/>
       <c r="E39" s="104"/>
       <c r="F39" s="104"/>
       <c r="G39" s="104"/>
@@ -2897,8 +2897,8 @@
       <c r="B40" s="25">
         <v>8</v>
       </c>
-      <c r="C40" s="28"/>
-      <c r="D40" s="28"/>
+      <c r="C40" s="32"/>
+      <c r="D40" s="32"/>
       <c r="E40" s="104"/>
       <c r="F40" s="104"/>
       <c r="G40" s="104"/>
@@ -2929,8 +2929,8 @@
       <c r="B41" s="25">
         <v>9</v>
       </c>
-      <c r="C41" s="28"/>
-      <c r="D41" s="28"/>
+      <c r="C41" s="32"/>
+      <c r="D41" s="32"/>
       <c r="E41" s="104"/>
       <c r="F41" s="104"/>
       <c r="G41" s="104"/>
@@ -2961,8 +2961,8 @@
       <c r="B42" s="25">
         <v>10</v>
       </c>
-      <c r="C42" s="28"/>
-      <c r="D42" s="28"/>
+      <c r="C42" s="32"/>
+      <c r="D42" s="32"/>
       <c r="E42" s="104"/>
       <c r="F42" s="104"/>
       <c r="G42" s="104"/>
@@ -2993,8 +2993,8 @@
       <c r="B43" s="25">
         <v>11</v>
       </c>
-      <c r="C43" s="28"/>
-      <c r="D43" s="28"/>
+      <c r="C43" s="32"/>
+      <c r="D43" s="32"/>
       <c r="E43" s="104"/>
       <c r="F43" s="104"/>
       <c r="G43" s="104"/>
@@ -3025,8 +3025,8 @@
       <c r="B44" s="25">
         <v>12</v>
       </c>
-      <c r="C44" s="28"/>
-      <c r="D44" s="28"/>
+      <c r="C44" s="32"/>
+      <c r="D44" s="32"/>
       <c r="E44" s="104"/>
       <c r="F44" s="104"/>
       <c r="G44" s="104"/>
@@ -3057,8 +3057,8 @@
       <c r="B45" s="25">
         <v>13</v>
       </c>
-      <c r="C45" s="28"/>
-      <c r="D45" s="28"/>
+      <c r="C45" s="32"/>
+      <c r="D45" s="32"/>
       <c r="E45" s="104"/>
       <c r="F45" s="104"/>
       <c r="G45" s="104"/>
@@ -3089,8 +3089,8 @@
       <c r="B46" s="25">
         <v>14</v>
       </c>
-      <c r="C46" s="28"/>
-      <c r="D46" s="28"/>
+      <c r="C46" s="32"/>
+      <c r="D46" s="32"/>
       <c r="E46" s="104"/>
       <c r="F46" s="104"/>
       <c r="G46" s="104"/>
@@ -3121,8 +3121,8 @@
       <c r="B47" s="25">
         <v>15</v>
       </c>
-      <c r="C47" s="28"/>
-      <c r="D47" s="28"/>
+      <c r="C47" s="32"/>
+      <c r="D47" s="32"/>
       <c r="E47" s="104"/>
       <c r="F47" s="104"/>
       <c r="G47" s="104"/>
@@ -3153,8 +3153,8 @@
       <c r="B48" s="25">
         <v>16</v>
       </c>
-      <c r="C48" s="28"/>
-      <c r="D48" s="28"/>
+      <c r="C48" s="32"/>
+      <c r="D48" s="32"/>
       <c r="E48" s="104"/>
       <c r="F48" s="104"/>
       <c r="G48" s="104"/>
@@ -3185,8 +3185,8 @@
       <c r="B49" s="25">
         <v>17</v>
       </c>
-      <c r="C49" s="28"/>
-      <c r="D49" s="28"/>
+      <c r="C49" s="32"/>
+      <c r="D49" s="32"/>
       <c r="E49" s="104"/>
       <c r="F49" s="104"/>
       <c r="G49" s="104"/>
@@ -3217,8 +3217,8 @@
       <c r="B50" s="25">
         <v>18</v>
       </c>
-      <c r="C50" s="28"/>
-      <c r="D50" s="28"/>
+      <c r="C50" s="32"/>
+      <c r="D50" s="32"/>
       <c r="E50" s="104"/>
       <c r="F50" s="104"/>
       <c r="G50" s="104"/>
@@ -3249,8 +3249,8 @@
       <c r="B51" s="25">
         <v>19</v>
       </c>
-      <c r="C51" s="28"/>
-      <c r="D51" s="28"/>
+      <c r="C51" s="32"/>
+      <c r="D51" s="32"/>
       <c r="E51" s="104"/>
       <c r="F51" s="104"/>
       <c r="G51" s="104"/>
@@ -3281,8 +3281,8 @@
       <c r="B52" s="25">
         <v>20</v>
       </c>
-      <c r="C52" s="28"/>
-      <c r="D52" s="28"/>
+      <c r="C52" s="32"/>
+      <c r="D52" s="32"/>
       <c r="E52" s="104"/>
       <c r="F52" s="104"/>
       <c r="G52" s="104"/>
@@ -3313,8 +3313,8 @@
       <c r="B53" s="25">
         <v>21</v>
       </c>
-      <c r="C53" s="28"/>
-      <c r="D53" s="28"/>
+      <c r="C53" s="32"/>
+      <c r="D53" s="32"/>
       <c r="E53" s="104"/>
       <c r="F53" s="104"/>
       <c r="G53" s="104"/>
@@ -3345,8 +3345,8 @@
       <c r="B54" s="25">
         <v>22</v>
       </c>
-      <c r="C54" s="28"/>
-      <c r="D54" s="28"/>
+      <c r="C54" s="32"/>
+      <c r="D54" s="32"/>
       <c r="E54" s="104"/>
       <c r="F54" s="104"/>
       <c r="G54" s="104"/>
@@ -3377,8 +3377,8 @@
       <c r="B55" s="25">
         <v>23</v>
       </c>
-      <c r="C55" s="28"/>
-      <c r="D55" s="28"/>
+      <c r="C55" s="32"/>
+      <c r="D55" s="32"/>
       <c r="E55" s="104"/>
       <c r="F55" s="104"/>
       <c r="G55" s="104"/>
@@ -3515,8 +3515,8 @@
       <c r="B60" s="25">
         <v>5</v>
       </c>
-      <c r="C60" s="26"/>
-      <c r="D60" s="28"/>
+      <c r="C60" s="30"/>
+      <c r="D60" s="32"/>
       <c r="E60" s="126"/>
       <c r="F60" s="126"/>
       <c r="G60" s="126"/>
@@ -3541,8 +3541,8 @@
       <c r="B61" s="25">
         <v>6</v>
       </c>
-      <c r="C61" s="26"/>
-      <c r="D61" s="28"/>
+      <c r="C61" s="30"/>
+      <c r="D61" s="32"/>
       <c r="E61" s="126"/>
       <c r="F61" s="126"/>
       <c r="G61" s="126"/>
@@ -3567,8 +3567,8 @@
       <c r="B62" s="25">
         <v>7</v>
       </c>
-      <c r="C62" s="26"/>
-      <c r="D62" s="28"/>
+      <c r="C62" s="30"/>
+      <c r="D62" s="32"/>
       <c r="E62" s="126"/>
       <c r="F62" s="126"/>
       <c r="G62" s="126"/>
@@ -3593,8 +3593,8 @@
       <c r="B63" s="25">
         <v>8</v>
       </c>
-      <c r="C63" s="26"/>
-      <c r="D63" s="28"/>
+      <c r="C63" s="30"/>
+      <c r="D63" s="32"/>
       <c r="E63" s="126"/>
       <c r="F63" s="126"/>
       <c r="G63" s="126"/>
@@ -3619,8 +3619,8 @@
       <c r="B64" s="25">
         <v>9</v>
       </c>
-      <c r="C64" s="28"/>
-      <c r="D64" s="28"/>
+      <c r="C64" s="32"/>
+      <c r="D64" s="32"/>
       <c r="E64" s="104"/>
       <c r="F64" s="104"/>
       <c r="G64" s="104"/>
@@ -3645,8 +3645,8 @@
       <c r="B65" s="25">
         <v>10</v>
       </c>
-      <c r="C65" s="28"/>
-      <c r="D65" s="28"/>
+      <c r="C65" s="32"/>
+      <c r="D65" s="32"/>
       <c r="E65" s="104"/>
       <c r="F65" s="104"/>
       <c r="G65" s="104"/>

</xml_diff>